<commit_message>
updated xpath in exel file
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_Test8.xlsx
+++ b/src/main/resources/Program_Field_Values_Test8.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24701"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A6D182B-6396-4FF3-9401-00562CA77ED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{219C241E-24AA-4D38-806E-DBFE50C5E726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="3" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="136">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -128,9 +128,6 @@
     <t>State governments;Independent school districts</t>
   </si>
   <si>
-    <t>ApplicationDueDate__c</t>
-  </si>
-  <si>
     <t>Financials</t>
   </si>
   <si>
@@ -441,6 +438,12 @@
   </si>
   <si>
     <t>fieldKPIsRequired__c</t>
+  </si>
+  <si>
+    <t>fieldApplicationDueDate__c</t>
+  </si>
+  <si>
+    <t>fieldProgram__c</t>
   </si>
 </sst>
 </file>
@@ -824,7 +827,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
@@ -835,7 +838,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>
@@ -846,7 +849,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>11</v>
@@ -857,7 +860,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
@@ -868,7 +871,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C6" t="s">
         <v>12</v>
@@ -879,7 +882,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
@@ -890,7 +893,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -901,7 +904,7 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C9">
         <v>365</v>
@@ -941,10 +944,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" t="s">
         <v>66</v>
-      </c>
-      <c r="C2" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -952,10 +955,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" t="s">
         <v>70</v>
-      </c>
-      <c r="C3" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -963,10 +966,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" t="s">
         <v>68</v>
-      </c>
-      <c r="C4" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1003,10 +1006,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1014,10 +1017,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" t="s">
         <v>70</v>
-      </c>
-      <c r="C3" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1025,10 +1028,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" t="s">
         <v>68</v>
-      </c>
-      <c r="C4" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1061,10 +1064,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1072,10 +1075,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3" t="s">
         <v>74</v>
-      </c>
-      <c r="C3" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1083,7 +1086,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1094,7 +1097,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C5">
         <v>3650</v>
@@ -1105,10 +1108,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" t="s">
         <v>78</v>
-      </c>
-      <c r="C6" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1116,10 +1119,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" t="s">
         <v>80</v>
-      </c>
-      <c r="C7" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1127,10 +1130,10 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>135</v>
       </c>
       <c r="C8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1138,10 +1141,10 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1219,7 +1222,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C6" t="s">
         <v>12</v>
@@ -1263,7 +1266,7 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
@@ -1285,7 +1288,7 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>8</v>
+        <v>130</v>
       </c>
       <c r="C12" t="s">
         <v>12</v>
@@ -1323,18 +1326,18 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C3">
         <v>3650</v>
@@ -1370,10 +1373,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C2" t="s">
         <v>94</v>
-      </c>
-      <c r="C2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1381,10 +1384,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1392,10 +1395,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C4" t="s">
         <v>97</v>
-      </c>
-      <c r="C4" t="s">
-        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -1429,7 +1432,7 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C2">
         <v>10</v>
@@ -1440,7 +1443,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C3">
         <v>20</v>
@@ -1451,10 +1454,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C4" t="s">
         <v>101</v>
-      </c>
-      <c r="C4" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1462,10 +1465,10 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1473,10 +1476,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C6" t="s">
         <v>104</v>
-      </c>
-      <c r="C6" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1484,10 +1487,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>105</v>
+      </c>
+      <c r="C7" t="s">
         <v>106</v>
-      </c>
-      <c r="C7" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1495,10 +1498,10 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1527,10 +1530,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1538,10 +1541,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1549,10 +1552,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1560,10 +1563,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1571,10 +1574,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1582,10 +1585,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1593,10 +1596,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1604,10 +1607,10 @@
         <v>3</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -1615,10 +1618,10 @@
         <v>3</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1692,7 +1695,7 @@
         <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1928,7 +1931,7 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>134</v>
       </c>
       <c r="C4">
         <v>20</v>
@@ -1936,10 +1939,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
         <v>31</v>
-      </c>
-      <c r="B5" t="s">
-        <v>32</v>
       </c>
       <c r="C5">
         <v>1000</v>
@@ -1947,10 +1950,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C6">
         <v>10000</v>
@@ -1958,10 +1961,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C7">
         <v>2</v>
@@ -1969,10 +1972,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C8">
         <v>10000</v>
@@ -2010,10 +2013,10 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" t="s">
         <v>37</v>
-      </c>
-      <c r="C2" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2021,54 +2024,54 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" t="s">
         <v>39</v>
-      </c>
-      <c r="C3" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
         <v>41</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>42</v>
-      </c>
-      <c r="C4" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" t="s">
         <v>44</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>45</v>
-      </c>
-      <c r="C5" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -2101,10 +2104,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" t="s">
         <v>50</v>
-      </c>
-      <c r="C2" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2112,10 +2115,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -2148,10 +2151,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" t="s">
         <v>52</v>
-      </c>
-      <c r="C2" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2159,10 +2162,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" t="s">
         <v>54</v>
-      </c>
-      <c r="C3" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2170,10 +2173,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" t="s">
         <v>56</v>
-      </c>
-      <c r="C4" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2181,10 +2184,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2192,10 +2195,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2203,10 +2206,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2214,10 +2217,10 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -2225,10 +2228,10 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -2236,10 +2239,10 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2247,10 +2250,10 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -2258,10 +2261,10 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -2294,10 +2297,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2305,10 +2308,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" t="s">
         <v>68</v>
-      </c>
-      <c r="C3" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2316,7 +2319,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -2327,7 +2330,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C5">
         <v>3650</v>
@@ -2338,10 +2341,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" t="s">
         <v>70</v>
-      </c>
-      <c r="C6" t="s">
-        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated changes as per comment
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_Test8.xlsx
+++ b/src/main/resources/Program_Field_Values_Test8.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25225"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58A4270C-0FCE-41D8-BE76-9463FD37B203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95862EEF-4160-4F94-BDB6-CDE4702A6A2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2820" yWindow="2820" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="3" r:id="rId1"/>

</xml_diff>